<commit_message>
Update example to reflect changes in TerrainCorrectionParameters
</commit_message>
<xml_diff>
--- a/examples/surveys/terrain_corrections/terrain_correction_results.xlsx
+++ b/examples/surveys/terrain_corrections/terrain_correction_results.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,48 +426,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>site_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>easting</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>northing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>dem_elevation</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem:topo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem:topo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>tcorr:total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -467,20 +474,17 @@
         <v>5424019.385</v>
       </c>
       <c r="D2" t="n">
-        <v>72.52800000000001</v>
+        <v>0.310109</v>
       </c>
       <c r="E2" t="n">
-        <v>0.310109</v>
+        <v>0.220958</v>
       </c>
       <c r="F2" t="n">
-        <v>1163.096392</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1163.406501</v>
+        <v>0.531067</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2.0</t>
         </is>
@@ -492,20 +496,17 @@
         <v>5424003.188</v>
       </c>
       <c r="D3" t="n">
-        <v>79.595</v>
+        <v>0.343483</v>
       </c>
       <c r="E3" t="n">
-        <v>0.343482</v>
+        <v>0.222331</v>
       </c>
       <c r="F3" t="n">
-        <v>1157.113712</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1157.457194</v>
+        <v>0.565814</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
@@ -517,20 +518,17 @@
         <v>5423994.639</v>
       </c>
       <c r="D4" t="n">
-        <v>87.16200000000001</v>
+        <v>0.427133</v>
       </c>
       <c r="E4" t="n">
-        <v>0.427133</v>
+        <v>0.226984</v>
       </c>
       <c r="F4" t="n">
-        <v>1157.673721</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1158.100854</v>
+        <v>0.6541169999999999</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
@@ -542,20 +540,17 @@
         <v>5423983.57</v>
       </c>
       <c r="D5" t="n">
-        <v>91.233</v>
+        <v>0.647508</v>
       </c>
       <c r="E5" t="n">
-        <v>0.647508</v>
+        <v>0.22687</v>
       </c>
       <c r="F5" t="n">
-        <v>1152.477911</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1153.125419</v>
+        <v>0.874378</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>7.0</t>
         </is>
@@ -567,20 +562,17 @@
         <v>5423979.679</v>
       </c>
       <c r="D6" t="n">
-        <v>80.488</v>
+        <v>0.620291</v>
       </c>
       <c r="E6" t="n">
-        <v>0.620291</v>
+        <v>0.214765</v>
       </c>
       <c r="F6" t="n">
-        <v>1153.24396</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1153.864251</v>
+        <v>0.835056</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>11.0</t>
         </is>
@@ -592,20 +584,17 @@
         <v>5423946.261</v>
       </c>
       <c r="D7" t="n">
-        <v>25.52</v>
+        <v>0.331787</v>
       </c>
       <c r="E7" t="n">
-        <v>0.331787</v>
+        <v>0.234568</v>
       </c>
       <c r="F7" t="n">
-        <v>1149.55242</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1149.884207</v>
+        <v>0.5663549999999999</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>12.0</t>
         </is>
@@ -617,20 +606,17 @@
         <v>5423941.581</v>
       </c>
       <c r="D8" t="n">
-        <v>20.604</v>
+        <v>0.316036</v>
       </c>
       <c r="E8" t="n">
-        <v>0.316036</v>
+        <v>0.240833</v>
       </c>
       <c r="F8" t="n">
-        <v>1150.044442</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1150.360478</v>
+        <v>0.5568689999999999</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>13.0</t>
         </is>
@@ -642,20 +628,17 @@
         <v>5423930.166</v>
       </c>
       <c r="D9" t="n">
-        <v>20.231</v>
+        <v>0.247567</v>
       </c>
       <c r="E9" t="n">
-        <v>0.247567</v>
+        <v>0.237406</v>
       </c>
       <c r="F9" t="n">
-        <v>1150.87634</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1151.123907</v>
+        <v>0.484973</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>14.0</t>
         </is>
@@ -667,20 +650,17 @@
         <v>5423912.414</v>
       </c>
       <c r="D10" t="n">
-        <v>19.983</v>
+        <v>0.203829</v>
       </c>
       <c r="E10" t="n">
-        <v>0.203829</v>
+        <v>0.237765</v>
       </c>
       <c r="F10" t="n">
-        <v>1148.18805</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1148.391879</v>
+        <v>0.441594</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>15.0</t>
         </is>
@@ -692,20 +672,17 @@
         <v>5423893.543</v>
       </c>
       <c r="D11" t="n">
-        <v>19.732</v>
+        <v>0.160821</v>
       </c>
       <c r="E11" t="n">
-        <v>0.160821</v>
+        <v>0.234413</v>
       </c>
       <c r="F11" t="n">
-        <v>1149.245957</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1149.406778</v>
+        <v>0.395234</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>16.0</t>
         </is>
@@ -717,20 +694,17 @@
         <v>5423881.772</v>
       </c>
       <c r="D12" t="n">
-        <v>19.433</v>
+        <v>0.139158</v>
       </c>
       <c r="E12" t="n">
-        <v>0.139158</v>
+        <v>0.232338</v>
       </c>
       <c r="F12" t="n">
-        <v>1149.955903</v>
-      </c>
-      <c r="G12" t="n">
-        <v>1150.095061</v>
+        <v>0.371496</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>17.0</t>
         </is>
@@ -742,20 +716,17 @@
         <v>5423865.674</v>
       </c>
       <c r="D13" t="n">
-        <v>18.919</v>
+        <v>0.118072</v>
       </c>
       <c r="E13" t="n">
-        <v>0.118072</v>
+        <v>0.229953</v>
       </c>
       <c r="F13" t="n">
-        <v>1150.91833</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1151.036402</v>
+        <v>0.348025</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>18.0</t>
         </is>
@@ -767,20 +738,17 @@
         <v>5423847.532</v>
       </c>
       <c r="D14" t="n">
-        <v>18.473</v>
+        <v>0.104907</v>
       </c>
       <c r="E14" t="n">
-        <v>0.104907</v>
+        <v>0.22924</v>
       </c>
       <c r="F14" t="n">
-        <v>1146.274014</v>
-      </c>
-      <c r="G14" t="n">
-        <v>1146.378921</v>
+        <v>0.334147</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>19.0</t>
         </is>
@@ -792,20 +760,17 @@
         <v>5423839.069</v>
       </c>
       <c r="D15" t="n">
-        <v>18.273</v>
+        <v>0.09851699999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>0.09851699999999999</v>
+        <v>0.228101</v>
       </c>
       <c r="F15" t="n">
-        <v>1146.767274</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1146.865791</v>
+        <v>0.326618</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
@@ -817,20 +782,17 @@
         <v>5423829.244</v>
       </c>
       <c r="D16" t="n">
-        <v>18.094</v>
+        <v>0.09096799999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>0.09096799999999999</v>
+        <v>0.226493</v>
       </c>
       <c r="F16" t="n">
-        <v>1147.37661</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1147.467578</v>
+        <v>0.317461</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>21.0</t>
         </is>
@@ -842,20 +804,17 @@
         <v>5423819.079</v>
       </c>
       <c r="D17" t="n">
-        <v>17.516</v>
+        <v>0.086273</v>
       </c>
       <c r="E17" t="n">
-        <v>0.086273</v>
+        <v>0.226092</v>
       </c>
       <c r="F17" t="n">
-        <v>1147.940063</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1148.026336</v>
+        <v>0.312365</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>22.0</t>
         </is>
@@ -867,20 +826,17 @@
         <v>5423812.404</v>
       </c>
       <c r="D18" t="n">
-        <v>17.434</v>
+        <v>0.082691</v>
       </c>
       <c r="E18" t="n">
-        <v>0.082691</v>
+        <v>0.225122</v>
       </c>
       <c r="F18" t="n">
-        <v>1148.335443</v>
-      </c>
-      <c r="G18" t="n">
-        <v>1148.418134</v>
+        <v>0.307813</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>23.0</t>
         </is>
@@ -892,20 +848,17 @@
         <v>5423803.196</v>
       </c>
       <c r="D19" t="n">
-        <v>16.945</v>
+        <v>0.079129</v>
       </c>
       <c r="E19" t="n">
-        <v>0.079129</v>
+        <v>0.224737</v>
       </c>
       <c r="F19" t="n">
-        <v>1148.850465</v>
-      </c>
-      <c r="G19" t="n">
-        <v>1148.929594</v>
+        <v>0.303866</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>24.0</t>
         </is>
@@ -917,20 +870,17 @@
         <v>5423795.166</v>
       </c>
       <c r="D20" t="n">
-        <v>16.63</v>
+        <v>0.076559</v>
       </c>
       <c r="E20" t="n">
-        <v>0.076559</v>
+        <v>0.224304</v>
       </c>
       <c r="F20" t="n">
-        <v>1149.284963</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1149.361522</v>
+        <v>0.300863</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>25.0</t>
         </is>
@@ -942,20 +892,17 @@
         <v>5423788.919</v>
       </c>
       <c r="D21" t="n">
-        <v>16.528</v>
+        <v>0.074139</v>
       </c>
       <c r="E21" t="n">
-        <v>0.074139</v>
+        <v>0.223571</v>
       </c>
       <c r="F21" t="n">
-        <v>1149.647335</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1149.721474</v>
+        <v>0.29771</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>26.0</t>
         </is>
@@ -967,20 +914,17 @@
         <v>5423782.989</v>
       </c>
       <c r="D22" t="n">
-        <v>16.158</v>
+        <v>0.07144200000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.07144200000000001</v>
+        <v>0.223822</v>
       </c>
       <c r="F22" t="n">
-        <v>1144.445002</v>
-      </c>
-      <c r="G22" t="n">
-        <v>1144.516444</v>
+        <v>0.295264</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>27.0</t>
         </is>
@@ -992,20 +936,17 @@
         <v>5423776.149</v>
       </c>
       <c r="D23" t="n">
-        <v>15.826</v>
+        <v>0.06893100000000001</v>
       </c>
       <c r="E23" t="n">
-        <v>0.06893100000000001</v>
+        <v>0.223279</v>
       </c>
       <c r="F23" t="n">
-        <v>1144.875932</v>
-      </c>
-      <c r="G23" t="n">
-        <v>1144.944863</v>
+        <v>0.29221</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>28.0</t>
         </is>
@@ -1017,20 +958,17 @@
         <v>5423771.029</v>
       </c>
       <c r="D24" t="n">
-        <v>15.556</v>
+        <v>0.06712600000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>0.06712600000000001</v>
+        <v>0.222898</v>
       </c>
       <c r="F24" t="n">
-        <v>1145.205486</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1145.272612</v>
+        <v>0.290024</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>29.0</t>
         </is>
@@ -1042,20 +980,17 @@
         <v>5423763.381</v>
       </c>
       <c r="D25" t="n">
-        <v>15.263</v>
+        <v>0.065011</v>
       </c>
       <c r="E25" t="n">
-        <v>0.065011</v>
+        <v>0.222318</v>
       </c>
       <c r="F25" t="n">
-        <v>1145.66626</v>
-      </c>
-      <c r="G25" t="n">
-        <v>1145.731271</v>
+        <v>0.287329</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>30.0</t>
         </is>
@@ -1067,20 +1002,17 @@
         <v>5423755.011</v>
       </c>
       <c r="D26" t="n">
-        <v>14.935</v>
+        <v>0.06313299999999999</v>
       </c>
       <c r="E26" t="n">
-        <v>0.06313299999999999</v>
+        <v>0.221822</v>
       </c>
       <c r="F26" t="n">
-        <v>1146.153871</v>
-      </c>
-      <c r="G26" t="n">
-        <v>1146.217004</v>
+        <v>0.284955</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>31.0</t>
         </is>
@@ -1092,20 +1024,17 @@
         <v>5423745.229</v>
       </c>
       <c r="D27" t="n">
-        <v>14.561</v>
+        <v>0.061826</v>
       </c>
       <c r="E27" t="n">
-        <v>0.061826</v>
+        <v>0.221555</v>
       </c>
       <c r="F27" t="n">
-        <v>1146.666168</v>
-      </c>
-      <c r="G27" t="n">
-        <v>1146.727994</v>
+        <v>0.283381</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>32.0</t>
         </is>
@@ -1117,20 +1046,17 @@
         <v>5423735.776</v>
       </c>
       <c r="D28" t="n">
-        <v>14.203</v>
+        <v>0.060161</v>
       </c>
       <c r="E28" t="n">
-        <v>0.060161</v>
+        <v>0.221097</v>
       </c>
       <c r="F28" t="n">
-        <v>1147.206551</v>
-      </c>
-      <c r="G28" t="n">
-        <v>1147.266712</v>
+        <v>0.281258</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>33.0</t>
         </is>
@@ -1142,20 +1068,17 @@
         <v>5423728.325</v>
       </c>
       <c r="D29" t="n">
-        <v>13.915</v>
+        <v>0.058523</v>
       </c>
       <c r="E29" t="n">
-        <v>0.058523</v>
+        <v>0.22056</v>
       </c>
       <c r="F29" t="n">
-        <v>1147.678805</v>
-      </c>
-      <c r="G29" t="n">
-        <v>1147.737328</v>
+        <v>0.279083</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>34.0</t>
         </is>
@@ -1167,20 +1090,17 @@
         <v>5423720.903</v>
       </c>
       <c r="D30" t="n">
-        <v>13.689</v>
+        <v>0.057046</v>
       </c>
       <c r="E30" t="n">
-        <v>0.057046</v>
+        <v>0.218033</v>
       </c>
       <c r="F30" t="n">
-        <v>1150.923228</v>
-      </c>
-      <c r="G30" t="n">
-        <v>1150.980274</v>
+        <v>0.275079</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>35.0</t>
         </is>
@@ -1192,20 +1112,17 @@
         <v>5423713.517</v>
       </c>
       <c r="D31" t="n">
-        <v>13.488</v>
+        <v>0.055731</v>
       </c>
       <c r="E31" t="n">
-        <v>0.055731</v>
+        <v>0.217547</v>
       </c>
       <c r="F31" t="n">
-        <v>1146.472259</v>
-      </c>
-      <c r="G31" t="n">
-        <v>1146.52799</v>
+        <v>0.273278</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>36.0</t>
         </is>
@@ -1217,20 +1134,17 @@
         <v>5423704.44</v>
       </c>
       <c r="D32" t="n">
-        <v>13.289</v>
+        <v>0.054448</v>
       </c>
       <c r="E32" t="n">
-        <v>0.054448</v>
+        <v>0.216792</v>
       </c>
       <c r="F32" t="n">
-        <v>1146.997188</v>
-      </c>
-      <c r="G32" t="n">
-        <v>1147.051636</v>
+        <v>0.27124</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>37.0</t>
         </is>
@@ -1242,20 +1156,17 @@
         <v>5423696.131</v>
       </c>
       <c r="D33" t="n">
-        <v>13.086</v>
+        <v>0.053288</v>
       </c>
       <c r="E33" t="n">
-        <v>0.053288</v>
+        <v>0.216127</v>
       </c>
       <c r="F33" t="n">
-        <v>1147.48728</v>
-      </c>
-      <c r="G33" t="n">
-        <v>1147.540568</v>
+        <v>0.269415</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>38.0</t>
         </is>
@@ -1267,20 +1178,17 @@
         <v>5423689.002</v>
       </c>
       <c r="D34" t="n">
-        <v>12.914</v>
+        <v>0.052243</v>
       </c>
       <c r="E34" t="n">
-        <v>0.052243</v>
+        <v>0.215508</v>
       </c>
       <c r="F34" t="n">
-        <v>1147.923552</v>
-      </c>
-      <c r="G34" t="n">
-        <v>1147.975795</v>
+        <v>0.267751</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>39.0</t>
         </is>
@@ -1292,20 +1200,17 @@
         <v>5423682.591</v>
       </c>
       <c r="D35" t="n">
-        <v>12.772</v>
+        <v>0.051314</v>
       </c>
       <c r="E35" t="n">
-        <v>0.051314</v>
+        <v>0.214931</v>
       </c>
       <c r="F35" t="n">
-        <v>1148.320536</v>
-      </c>
-      <c r="G35" t="n">
-        <v>1148.37185</v>
+        <v>0.266245</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>40.0</t>
         </is>
@@ -1317,20 +1222,17 @@
         <v>5423675.873</v>
       </c>
       <c r="D36" t="n">
-        <v>12.617</v>
+        <v>0.050535</v>
       </c>
       <c r="E36" t="n">
-        <v>0.050535</v>
+        <v>0.214439</v>
       </c>
       <c r="F36" t="n">
-        <v>1148.716535</v>
-      </c>
-      <c r="G36" t="n">
-        <v>1148.76707</v>
+        <v>0.264974</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>41.0</t>
         </is>
@@ -1342,20 +1244,17 @@
         <v>5423669.103</v>
       </c>
       <c r="D37" t="n">
-        <v>12.658</v>
+        <v>0.04952</v>
       </c>
       <c r="E37" t="n">
-        <v>0.04952</v>
+        <v>0.213551</v>
       </c>
       <c r="F37" t="n">
-        <v>1149.12765</v>
-      </c>
-      <c r="G37" t="n">
-        <v>1149.17717</v>
+        <v>0.263071</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>42.0</t>
         </is>
@@ -1367,20 +1266,17 @@
         <v>5423662.146</v>
       </c>
       <c r="D38" t="n">
-        <v>12.292</v>
+        <v>0.042929</v>
       </c>
       <c r="E38" t="n">
-        <v>0.042929</v>
+        <v>0.211208</v>
       </c>
       <c r="F38" t="n">
-        <v>1145.925814</v>
-      </c>
-      <c r="G38" t="n">
-        <v>1145.968743</v>
+        <v>0.254137</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>43.0</t>
         </is>
@@ -1392,20 +1288,17 @@
         <v>5423666.1</v>
       </c>
       <c r="D39" t="n">
-        <v>12.169</v>
+        <v>0.041881</v>
       </c>
       <c r="E39" t="n">
-        <v>0.041881</v>
+        <v>0.210513</v>
       </c>
       <c r="F39" t="n">
-        <v>1146.076681</v>
-      </c>
-      <c r="G39" t="n">
-        <v>1146.118562</v>
+        <v>0.252394</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>44.0</t>
         </is>
@@ -1417,20 +1310,17 @@
         <v>5423670.24</v>
       </c>
       <c r="D40" t="n">
-        <v>12.316</v>
+        <v>0.040654</v>
       </c>
       <c r="E40" t="n">
-        <v>0.040654</v>
+        <v>0.209475</v>
       </c>
       <c r="F40" t="n">
-        <v>1146.195104</v>
-      </c>
-      <c r="G40" t="n">
-        <v>1146.235758</v>
+        <v>0.250129</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>45.0</t>
         </is>
@@ -1442,20 +1332,17 @@
         <v>5423663.578</v>
       </c>
       <c r="D41" t="n">
-        <v>12.112</v>
+        <v>0.040381</v>
       </c>
       <c r="E41" t="n">
-        <v>0.040381</v>
+        <v>0.209162</v>
       </c>
       <c r="F41" t="n">
-        <v>1146.606696</v>
-      </c>
-      <c r="G41" t="n">
-        <v>1146.647077</v>
+        <v>0.249543</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>46.0</t>
         </is>
@@ -1467,20 +1354,17 @@
         <v>5423654.783</v>
       </c>
       <c r="D42" t="n">
-        <v>11.724</v>
+        <v>0.039571</v>
       </c>
       <c r="E42" t="n">
-        <v>0.039571</v>
+        <v>0.211416</v>
       </c>
       <c r="F42" t="n">
-        <v>1141.79258</v>
-      </c>
-      <c r="G42" t="n">
-        <v>1141.832151</v>
+        <v>0.250987</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>47.0</t>
         </is>
@@ -1492,20 +1376,17 @@
         <v>5423646.209</v>
       </c>
       <c r="D43" t="n">
-        <v>11.364</v>
+        <v>0.039069</v>
       </c>
       <c r="E43" t="n">
-        <v>0.039069</v>
+        <v>0.210382</v>
       </c>
       <c r="F43" t="n">
-        <v>1142.558517</v>
-      </c>
-      <c r="G43" t="n">
-        <v>1142.597586</v>
+        <v>0.249451</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>48.0</t>
         </is>
@@ -1517,20 +1398,17 @@
         <v>5423637.96</v>
       </c>
       <c r="D44" t="n">
-        <v>11.392</v>
+        <v>0.038481</v>
       </c>
       <c r="E44" t="n">
-        <v>0.038481</v>
+        <v>0.208753</v>
       </c>
       <c r="F44" t="n">
-        <v>1143.322171</v>
-      </c>
-      <c r="G44" t="n">
-        <v>1143.360652</v>
+        <v>0.247234</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>49.0</t>
         </is>
@@ -1542,20 +1420,17 @@
         <v>5423630.178</v>
       </c>
       <c r="D45" t="n">
-        <v>11.537</v>
+        <v>0.038064</v>
       </c>
       <c r="E45" t="n">
-        <v>0.038064</v>
+        <v>0.207043</v>
       </c>
       <c r="F45" t="n">
-        <v>1144.075914</v>
-      </c>
-      <c r="G45" t="n">
-        <v>1144.113978</v>
+        <v>0.245107</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>50.0</t>
         </is>
@@ -1567,20 +1442,17 @@
         <v>5423623.396</v>
       </c>
       <c r="D46" t="n">
-        <v>12.049</v>
+        <v>0.03725</v>
       </c>
       <c r="E46" t="n">
-        <v>0.03725</v>
+        <v>0.208955</v>
       </c>
       <c r="F46" t="n">
-        <v>1137.777419</v>
-      </c>
-      <c r="G46" t="n">
-        <v>1137.814669</v>
+        <v>0.246205</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>51.0</t>
         </is>
@@ -1592,20 +1464,17 @@
         <v>5423605.784</v>
       </c>
       <c r="D47" t="n">
-        <v>12.726</v>
+        <v>0.036582</v>
       </c>
       <c r="E47" t="n">
-        <v>0.036582</v>
+        <v>0.206321</v>
       </c>
       <c r="F47" t="n">
-        <v>1138.777615</v>
-      </c>
-      <c r="G47" t="n">
-        <v>1138.814197</v>
+        <v>0.242903</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>52.0</t>
         </is>
@@ -1617,20 +1486,17 @@
         <v>5423578.714</v>
       </c>
       <c r="D48" t="n">
-        <v>13.636</v>
+        <v>0.036332</v>
       </c>
       <c r="E48" t="n">
-        <v>0.036332</v>
+        <v>0.202915</v>
       </c>
       <c r="F48" t="n">
-        <v>1140.280581</v>
-      </c>
-      <c r="G48" t="n">
-        <v>1140.316913</v>
+        <v>0.239247</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>53.0</t>
         </is>
@@ -1642,20 +1508,17 @@
         <v>5423570.902</v>
       </c>
       <c r="D49" t="n">
-        <v>14.178</v>
+        <v>0.036215</v>
       </c>
       <c r="E49" t="n">
-        <v>0.036215</v>
+        <v>0.201214</v>
       </c>
       <c r="F49" t="n">
-        <v>1140.859523</v>
-      </c>
-      <c r="G49" t="n">
-        <v>1140.895738</v>
+        <v>0.237429</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>54.0</t>
         </is>
@@ -1667,20 +1530,17 @@
         <v>5423549.699</v>
       </c>
       <c r="D50" t="n">
-        <v>14.634</v>
+        <v>0.036649</v>
       </c>
       <c r="E50" t="n">
-        <v>0.036649</v>
+        <v>0.202861</v>
       </c>
       <c r="F50" t="n">
-        <v>1135.292953</v>
-      </c>
-      <c r="G50" t="n">
-        <v>1135.329602</v>
+        <v>0.23951</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>55.0</t>
         </is>
@@ -1692,20 +1552,17 @@
         <v>5423533.188</v>
       </c>
       <c r="D51" t="n">
-        <v>15.664</v>
+        <v>0.037059</v>
       </c>
       <c r="E51" t="n">
-        <v>0.037059</v>
+        <v>0.199738</v>
       </c>
       <c r="F51" t="n">
-        <v>1136.339131</v>
-      </c>
-      <c r="G51" t="n">
-        <v>1136.37619</v>
+        <v>0.236797</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>56.0</t>
         </is>
@@ -1717,20 +1574,17 @@
         <v>5423533.838</v>
       </c>
       <c r="D52" t="n">
-        <v>16.684</v>
+        <v>0.037365</v>
       </c>
       <c r="E52" t="n">
-        <v>0.037365</v>
+        <v>0.19725</v>
       </c>
       <c r="F52" t="n">
-        <v>1136.732067</v>
-      </c>
-      <c r="G52" t="n">
-        <v>1136.769432</v>
+        <v>0.234615</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>57.0</t>
         </is>
@@ -1742,20 +1596,17 @@
         <v>5423534.941</v>
       </c>
       <c r="D53" t="n">
-        <v>17.682</v>
+        <v>0.037925</v>
       </c>
       <c r="E53" t="n">
-        <v>0.037925</v>
+        <v>0.195083</v>
       </c>
       <c r="F53" t="n">
-        <v>1137.082992</v>
-      </c>
-      <c r="G53" t="n">
-        <v>1137.120917</v>
+        <v>0.233008</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="1" t="inlineStr">
         <is>
           <t>58.0</t>
         </is>
@@ -1767,20 +1618,17 @@
         <v>5423536.254</v>
       </c>
       <c r="D54" t="n">
-        <v>18.461</v>
+        <v>0.038907</v>
       </c>
       <c r="E54" t="n">
-        <v>0.038907</v>
+        <v>0.194702</v>
       </c>
       <c r="F54" t="n">
-        <v>1130.489371</v>
-      </c>
-      <c r="G54" t="n">
-        <v>1130.528278</v>
+        <v>0.233609</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="1" t="inlineStr">
         <is>
           <t>59.0</t>
         </is>
@@ -1792,20 +1640,17 @@
         <v>5423537.81</v>
       </c>
       <c r="D55" t="n">
-        <v>19.042</v>
+        <v>0.040225</v>
       </c>
       <c r="E55" t="n">
-        <v>0.040225</v>
+        <v>0.193267</v>
       </c>
       <c r="F55" t="n">
-        <v>1130.750954</v>
-      </c>
-      <c r="G55" t="n">
-        <v>1130.791179</v>
+        <v>0.233492</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="1" t="inlineStr">
         <is>
           <t>60.0</t>
         </is>
@@ -1817,20 +1662,17 @@
         <v>5423538.394</v>
       </c>
       <c r="D56" t="n">
-        <v>19.643</v>
+        <v>0.042278</v>
       </c>
       <c r="E56" t="n">
-        <v>0.042278</v>
+        <v>0.191844</v>
       </c>
       <c r="F56" t="n">
-        <v>1131.106958</v>
-      </c>
-      <c r="G56" t="n">
-        <v>1131.149236</v>
+        <v>0.234122</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="1" t="inlineStr">
         <is>
           <t>61.0</t>
         </is>
@@ -1842,20 +1684,17 @@
         <v>5423539.853</v>
       </c>
       <c r="D57" t="n">
-        <v>19.984</v>
+        <v>0.044228</v>
       </c>
       <c r="E57" t="n">
-        <v>0.044228</v>
+        <v>0.190995</v>
       </c>
       <c r="F57" t="n">
-        <v>1131.364441</v>
-      </c>
-      <c r="G57" t="n">
-        <v>1131.408669</v>
+        <v>0.235223</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="1" t="inlineStr">
         <is>
           <t>62.0</t>
         </is>
@@ -1867,20 +1706,17 @@
         <v>5423541.02</v>
       </c>
       <c r="D58" t="n">
-        <v>20.039</v>
+        <v>0.047037</v>
       </c>
       <c r="E58" t="n">
-        <v>0.047037</v>
+        <v>0.191</v>
       </c>
       <c r="F58" t="n">
-        <v>1125.028146</v>
-      </c>
-      <c r="G58" t="n">
-        <v>1125.075183</v>
+        <v>0.238037</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="1" t="inlineStr">
         <is>
           <t>63.0</t>
         </is>
@@ -1892,20 +1728,17 @@
         <v>5423542.528</v>
       </c>
       <c r="D59" t="n">
-        <v>20.066</v>
+        <v>0.050317</v>
       </c>
       <c r="E59" t="n">
-        <v>0.050317</v>
+        <v>0.190592</v>
       </c>
       <c r="F59" t="n">
-        <v>1125.193471</v>
-      </c>
-      <c r="G59" t="n">
-        <v>1125.243788</v>
+        <v>0.240909</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="1" t="inlineStr">
         <is>
           <t>64.0</t>
         </is>
@@ -1917,20 +1750,17 @@
         <v>5423543.501</v>
       </c>
       <c r="D60" t="n">
-        <v>20.049</v>
+        <v>0.054991</v>
       </c>
       <c r="E60" t="n">
-        <v>0.054991</v>
+        <v>0.190264</v>
       </c>
       <c r="F60" t="n">
-        <v>1125.423596</v>
-      </c>
-      <c r="G60" t="n">
-        <v>1125.478587</v>
+        <v>0.245255</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="1" t="inlineStr">
         <is>
           <t>65.0</t>
         </is>
@@ -1942,20 +1772,17 @@
         <v>5423544.668</v>
       </c>
       <c r="D61" t="n">
-        <v>19.991</v>
+        <v>0.05902</v>
       </c>
       <c r="E61" t="n">
-        <v>0.05902</v>
+        <v>0.190144</v>
       </c>
       <c r="F61" t="n">
-        <v>1125.58246</v>
-      </c>
-      <c r="G61" t="n">
-        <v>1125.64148</v>
+        <v>0.249164</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="1" t="inlineStr">
         <is>
           <t>66.0</t>
         </is>
@@ -1967,20 +1794,17 @@
         <v>5423532.22</v>
       </c>
       <c r="D62" t="n">
-        <v>20.046</v>
+        <v>0.065661</v>
       </c>
       <c r="E62" t="n">
-        <v>0.065661</v>
+        <v>0.19034</v>
       </c>
       <c r="F62" t="n">
-        <v>1118.8642</v>
-      </c>
-      <c r="G62" t="n">
-        <v>1118.929861</v>
+        <v>0.256001</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="1" t="inlineStr">
         <is>
           <t>67.0</t>
         </is>
@@ -1992,20 +1816,17 @@
         <v>5423527.204</v>
       </c>
       <c r="D63" t="n">
-        <v>19.941</v>
+        <v>0.073518</v>
       </c>
       <c r="E63" t="n">
-        <v>0.073518</v>
+        <v>0.190298</v>
       </c>
       <c r="F63" t="n">
-        <v>1119.109843</v>
-      </c>
-      <c r="G63" t="n">
-        <v>1119.183361</v>
+        <v>0.263816</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="1" t="inlineStr">
         <is>
           <t>68.0</t>
         </is>
@@ -2017,20 +1838,17 @@
         <v>5423540.219</v>
       </c>
       <c r="D64" t="n">
-        <v>19.94</v>
+        <v>0.082494</v>
       </c>
       <c r="E64" t="n">
-        <v>0.082494</v>
+        <v>0.190315</v>
       </c>
       <c r="F64" t="n">
-        <v>1118.817622</v>
-      </c>
-      <c r="G64" t="n">
-        <v>1118.900116</v>
+        <v>0.272809</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="1" t="inlineStr">
         <is>
           <t>69.0</t>
         </is>
@@ -2042,20 +1860,17 @@
         <v>5423511.1642151</v>
       </c>
       <c r="D65" t="n">
-        <v>20.018</v>
+        <v>0.09715799999999999</v>
       </c>
       <c r="E65" t="n">
-        <v>0.09715799999999999</v>
+        <v>0.189992</v>
       </c>
       <c r="F65" t="n">
-        <v>1120.824905</v>
-      </c>
-      <c r="G65" t="n">
-        <v>1120.922063</v>
+        <v>0.28715</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="1" t="inlineStr">
         <is>
           <t>70.0</t>
         </is>
@@ -2067,20 +1882,17 @@
         <v>5423464.549959657</v>
       </c>
       <c r="D66" t="n">
-        <v>20.002</v>
+        <v>0.144643</v>
       </c>
       <c r="E66" t="n">
-        <v>0.144643</v>
+        <v>0.190476</v>
       </c>
       <c r="F66" t="n">
-        <v>1115.152852</v>
-      </c>
-      <c r="G66" t="n">
-        <v>1115.297495</v>
+        <v>0.335119</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="1" t="inlineStr">
         <is>
           <t>72.0</t>
         </is>
@@ -2092,20 +1904,17 @@
         <v>5423423.716027891</v>
       </c>
       <c r="D67" t="n">
-        <v>20.168</v>
+        <v>0.293752</v>
       </c>
       <c r="E67" t="n">
-        <v>0.293752</v>
+        <v>0.19128</v>
       </c>
       <c r="F67" t="n">
-        <v>1108.815234</v>
-      </c>
-      <c r="G67" t="n">
-        <v>1109.108986</v>
+        <v>0.485032</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="1" t="inlineStr">
         <is>
           <t>74.0</t>
         </is>
@@ -2117,20 +1926,17 @@
         <v>5423348.944608703</v>
       </c>
       <c r="D68" t="n">
-        <v>46.332</v>
+        <v>0.38862</v>
       </c>
       <c r="E68" t="n">
-        <v>0.38862</v>
+        <v>0.18169</v>
       </c>
       <c r="F68" t="n">
-        <v>1110.392378</v>
-      </c>
-      <c r="G68" t="n">
-        <v>1110.780998</v>
+        <v>0.57031</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="1" t="inlineStr">
         <is>
           <t>75.0</t>
         </is>
@@ -2142,20 +1948,17 @@
         <v>5423312.76796278</v>
       </c>
       <c r="D69" t="n">
-        <v>91.633</v>
+        <v>0.89672</v>
       </c>
       <c r="E69" t="n">
-        <v>0.89672</v>
+        <v>0.24234</v>
       </c>
       <c r="F69" t="n">
-        <v>1103.452197</v>
-      </c>
-      <c r="G69" t="n">
-        <v>1104.348917</v>
+        <v>1.13906</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="1" t="inlineStr">
         <is>
           <t>77.0</t>
         </is>
@@ -2167,20 +1970,17 @@
         <v>5423241.179389093</v>
       </c>
       <c r="D70" t="n">
-        <v>119.49</v>
+        <v>1.693565</v>
       </c>
       <c r="E70" t="n">
-        <v>1.693565</v>
+        <v>0.329467</v>
       </c>
       <c r="F70" t="n">
-        <v>1094.541024</v>
-      </c>
-      <c r="G70" t="n">
-        <v>1096.234589</v>
+        <v>2.023032</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="1" t="inlineStr">
         <is>
           <t>78.0</t>
         </is>
@@ -2192,20 +1992,17 @@
         <v>5423249.218</v>
       </c>
       <c r="D71" t="n">
-        <v>122.445</v>
+        <v>1.9137</v>
       </c>
       <c r="E71" t="n">
-        <v>1.9137</v>
+        <v>0.340762</v>
       </c>
       <c r="F71" t="n">
-        <v>1093.868106</v>
-      </c>
-      <c r="G71" t="n">
-        <v>1095.781806</v>
+        <v>2.254462</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="1" t="inlineStr">
         <is>
           <t>79.0</t>
         </is>
@@ -2217,20 +2014,17 @@
         <v>5423228.542</v>
       </c>
       <c r="D72" t="n">
-        <v>104.524</v>
+        <v>1.382242</v>
       </c>
       <c r="E72" t="n">
-        <v>1.382242</v>
+        <v>0.279542</v>
       </c>
       <c r="F72" t="n">
-        <v>1093.819956</v>
-      </c>
-      <c r="G72" t="n">
-        <v>1095.202198</v>
+        <v>1.661784</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="1" t="inlineStr">
         <is>
           <t>80.0</t>
         </is>
@@ -2242,20 +2036,17 @@
         <v>5423269.479</v>
       </c>
       <c r="D73" t="n">
-        <v>76.593</v>
+        <v>0.802502</v>
       </c>
       <c r="E73" t="n">
-        <v>0.802502</v>
+        <v>0.214845</v>
       </c>
       <c r="F73" t="n">
-        <v>1092.376371</v>
-      </c>
-      <c r="G73" t="n">
-        <v>1093.178873</v>
+        <v>1.017347</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="1" t="inlineStr">
         <is>
           <t>82.0</t>
         </is>
@@ -2267,20 +2058,17 @@
         <v>5423143.827</v>
       </c>
       <c r="D74" t="n">
-        <v>102.751</v>
+        <v>1.71337</v>
       </c>
       <c r="E74" t="n">
-        <v>1.71337</v>
+        <v>0.274704</v>
       </c>
       <c r="F74" t="n">
-        <v>1084.150718</v>
-      </c>
-      <c r="G74" t="n">
-        <v>1085.864088</v>
+        <v>1.988074</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="1" t="inlineStr">
         <is>
           <t>84.0</t>
         </is>
@@ -2292,20 +2080,17 @@
         <v>5423095.066</v>
       </c>
       <c r="D75" t="n">
-        <v>47.193</v>
+        <v>0.554856</v>
       </c>
       <c r="E75" t="n">
-        <v>0.554856</v>
+        <v>0.189866</v>
       </c>
       <c r="F75" t="n">
-        <v>1086.021937</v>
-      </c>
-      <c r="G75" t="n">
-        <v>1086.576793</v>
+        <v>0.744722</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="1" t="inlineStr">
         <is>
           <t>86.5</t>
         </is>
@@ -2317,20 +2102,17 @@
         <v>5423062.479</v>
       </c>
       <c r="D76" t="n">
-        <v>34.785</v>
+        <v>0.399428</v>
       </c>
       <c r="E76" t="n">
-        <v>0.399428</v>
+        <v>0.193444</v>
       </c>
       <c r="F76" t="n">
-        <v>1075.40116</v>
-      </c>
-      <c r="G76" t="n">
-        <v>1075.800588</v>
+        <v>0.5928720000000001</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="1" t="inlineStr">
         <is>
           <t>88.0</t>
         </is>
@@ -2342,20 +2124,17 @@
         <v>5423120.017</v>
       </c>
       <c r="D77" t="n">
-        <v>54.137</v>
+        <v>0.628498</v>
       </c>
       <c r="E77" t="n">
-        <v>0.628498</v>
+        <v>0.195638</v>
       </c>
       <c r="F77" t="n">
-        <v>1072.271111</v>
-      </c>
-      <c r="G77" t="n">
-        <v>1072.899609</v>
+        <v>0.824136</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="1" t="inlineStr">
         <is>
           <t>91.0</t>
         </is>
@@ -2367,20 +2146,17 @@
         <v>5423108.621</v>
       </c>
       <c r="D78" t="n">
-        <v>29.462</v>
+        <v>0.220937</v>
       </c>
       <c r="E78" t="n">
-        <v>0.220937</v>
+        <v>0.20402</v>
       </c>
       <c r="F78" t="n">
-        <v>1060.714972</v>
-      </c>
-      <c r="G78" t="n">
-        <v>1060.935909</v>
+        <v>0.424957</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="1" t="inlineStr">
         <is>
           <t>92.5</t>
         </is>
@@ -2392,20 +2168,17 @@
         <v>5423074.392</v>
       </c>
       <c r="D79" t="n">
-        <v>39.395</v>
+        <v>0.391791</v>
       </c>
       <c r="E79" t="n">
-        <v>0.391791</v>
+        <v>0.200753</v>
       </c>
       <c r="F79" t="n">
-        <v>1059.894669</v>
-      </c>
-      <c r="G79" t="n">
-        <v>1060.28646</v>
+        <v>0.592544</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="1" t="inlineStr">
         <is>
           <t>415.0</t>
         </is>
@@ -2417,20 +2190,17 @@
         <v>5423667.314</v>
       </c>
       <c r="D80" t="n">
-        <v>12.533</v>
+        <v>0.048488</v>
       </c>
       <c r="E80" t="n">
-        <v>0.048488</v>
+        <v>0.212964</v>
       </c>
       <c r="F80" t="n">
-        <v>1149.396266</v>
-      </c>
-      <c r="G80" t="n">
-        <v>1149.444754</v>
+        <v>0.261452</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="1" t="inlineStr">
         <is>
           <t>41.8</t>
         </is>
@@ -2442,20 +2212,17 @@
         <v>5423673.695</v>
       </c>
       <c r="D81" t="n">
-        <v>12.623</v>
+        <v>0.043773</v>
       </c>
       <c r="E81" t="n">
-        <v>0.043773</v>
+        <v>0.211941</v>
       </c>
       <c r="F81" t="n">
-        <v>1145.206929</v>
-      </c>
-      <c r="G81" t="n">
-        <v>1145.250702</v>
+        <v>0.255714</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="1" t="inlineStr">
         <is>
           <t>45.1</t>
         </is>
@@ -2467,20 +2234,17 @@
         <v>5423661.689</v>
       </c>
       <c r="D82" t="n">
-        <v>12.112</v>
+        <v>0.040403</v>
       </c>
       <c r="E82" t="n">
-        <v>0.040403</v>
+        <v>0.209139</v>
       </c>
       <c r="F82" t="n">
-        <v>1146.66914</v>
-      </c>
-      <c r="G82" t="n">
-        <v>1146.709543</v>
+        <v>0.249542</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="1" t="inlineStr">
         <is>
           <t>46.1</t>
         </is>
@@ -2492,20 +2256,17 @@
         <v>5423653.804</v>
       </c>
       <c r="D83" t="n">
-        <v>11.724</v>
+        <v>0.039577</v>
       </c>
       <c r="E83" t="n">
-        <v>0.039577</v>
+        <v>0.211406</v>
       </c>
       <c r="F83" t="n">
-        <v>1141.825005</v>
-      </c>
-      <c r="G83" t="n">
-        <v>1141.864582</v>
+        <v>0.250983</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="1" t="inlineStr">
         <is>
           <t>47.1</t>
         </is>
@@ -2517,20 +2278,17 @@
         <v>5423645.53</v>
       </c>
       <c r="D84" t="n">
-        <v>11.362</v>
+        <v>0.039175</v>
       </c>
       <c r="E84" t="n">
-        <v>0.039175</v>
+        <v>0.21038</v>
       </c>
       <c r="F84" t="n">
-        <v>1142.58017</v>
-      </c>
-      <c r="G84" t="n">
-        <v>1142.619345</v>
+        <v>0.249555</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="1" t="inlineStr">
         <is>
           <t>48.1</t>
         </is>
@@ -2542,20 +2300,17 @@
         <v>5423637.474</v>
       </c>
       <c r="D85" t="n">
-        <v>11.392</v>
+        <v>0.038483</v>
       </c>
       <c r="E85" t="n">
-        <v>0.038483</v>
+        <v>0.208745</v>
       </c>
       <c r="F85" t="n">
-        <v>1143.338904</v>
-      </c>
-      <c r="G85" t="n">
-        <v>1143.377387</v>
+        <v>0.247228</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="1" t="inlineStr">
         <is>
           <t>49.1</t>
         </is>
@@ -2567,20 +2322,17 @@
         <v>5423629.267</v>
       </c>
       <c r="D86" t="n">
-        <v>11.537</v>
+        <v>0.038068</v>
       </c>
       <c r="E86" t="n">
-        <v>0.038068</v>
+        <v>0.207033</v>
       </c>
       <c r="F86" t="n">
-        <v>1144.106079</v>
-      </c>
-      <c r="G86" t="n">
-        <v>1144.144147</v>
+        <v>0.245101</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="1" t="inlineStr">
         <is>
           <t>50.1</t>
         </is>
@@ -2592,16 +2344,13 @@
         <v>5423621.661</v>
       </c>
       <c r="D87" t="n">
-        <v>12.049</v>
+        <v>0.037263</v>
       </c>
       <c r="E87" t="n">
-        <v>0.037263</v>
+        <v>0.208941</v>
       </c>
       <c r="F87" t="n">
-        <v>1137.83377</v>
-      </c>
-      <c r="G87" t="n">
-        <v>1137.871033</v>
+        <v>0.246204</v>
       </c>
     </row>
   </sheetData>
@@ -2615,28 +2364,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>zone</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parameter</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>parameter_value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2653,7 +2402,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2668,7 +2417,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2683,7 +2432,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2698,7 +2447,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2713,7 +2462,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2728,7 +2477,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2745,7 +2494,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2757,12 +2506,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>d:\dropbox\git\gsolve\examples\surveys\terrain_corrections\Wellington8m_Land.tif</t>
+          <t>/home/adrianmb/Documents/projects/gsolve/examples/surveys/terrain_corrections/Wellington8m_Land.tif</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2775,7 +2524,7 @@
       <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2790,7 +2539,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>tcorr:8m_dem</t>
         </is>
@@ -2805,172 +2554,308 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:8m_dem</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>site_height_field</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>dem_elevation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:8m_dem</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>site_easting_field</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>easting</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:8m_dem</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>site_northing_field</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>northing</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:8m_dem</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>harmonica</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>200m_dem</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>min_dist</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C18" t="n">
         <v>2160</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>max_dist</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C19" t="n">
         <v>21900</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>terrain_density</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C20" t="n">
         <v>2670</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>water_density</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C21" t="n">
         <v>1030</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>sea_level_elevation</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C22" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>distance_mask_type</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>radial</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>dem_source</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>d:\dropbox\git\gsolve\examples\surveys\terrain_corrections\wellington200m_Land.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>/home/adrianmb/Documents/projects/gsolve/examples/surveys/terrain_corrections/Wellington200m_Land.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>density_dataset_source</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>compute_topography</t>
         </is>
       </c>
-      <c r="C22" t="b">
+      <c r="C26" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>compute_bathymetry</t>
         </is>
       </c>
-      <c r="C23" t="b">
+      <c r="C27" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:200m_dem</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>site_height_field</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>dem_elevation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:200m_dem</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>site_easting_field</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>easting</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:200m_dem</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>site_northing_field</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>northing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>tcorr:200m_dem</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>harmonica</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tcorrs: update example, output include new height columns
</commit_message>
<xml_diff>
--- a/examples/surveys/terrain_corrections/terrain_correction_results.xlsx
+++ b/examples/surveys/terrain_corrections/terrain_correction_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,15 +447,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>elev:8m_dem</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>elev:200m_dem</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>tcorr:8m_dem:topo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tcorr:200m_dem:topo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>tcorr:total</t>
         </is>
@@ -474,12 +484,18 @@
         <v>5424019.385</v>
       </c>
       <c r="D2" t="n">
+        <v>72.52800000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>72.52800000000001</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.310109</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>0.220958</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>0.531067</v>
       </c>
     </row>
@@ -496,12 +512,18 @@
         <v>5424003.188</v>
       </c>
       <c r="D3" t="n">
+        <v>79.595001</v>
+      </c>
+      <c r="E3" t="n">
+        <v>79.595001</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.343483</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>0.222331</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>0.565814</v>
       </c>
     </row>
@@ -518,12 +540,18 @@
         <v>5423994.639</v>
       </c>
       <c r="D4" t="n">
+        <v>87.162003</v>
+      </c>
+      <c r="E4" t="n">
+        <v>87.162003</v>
+      </c>
+      <c r="F4" t="n">
         <v>0.427133</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>0.226984</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>0.6541169999999999</v>
       </c>
     </row>
@@ -540,12 +568,18 @@
         <v>5423983.57</v>
       </c>
       <c r="D5" t="n">
+        <v>91.233002</v>
+      </c>
+      <c r="E5" t="n">
+        <v>91.233002</v>
+      </c>
+      <c r="F5" t="n">
         <v>0.647508</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>0.22687</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>0.874378</v>
       </c>
     </row>
@@ -562,12 +596,18 @@
         <v>5423979.679</v>
       </c>
       <c r="D6" t="n">
+        <v>80.487999</v>
+      </c>
+      <c r="E6" t="n">
+        <v>80.487999</v>
+      </c>
+      <c r="F6" t="n">
         <v>0.620291</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>0.214765</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>0.835056</v>
       </c>
     </row>
@@ -584,12 +624,18 @@
         <v>5423946.261</v>
       </c>
       <c r="D7" t="n">
+        <v>25.52</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25.52</v>
+      </c>
+      <c r="F7" t="n">
         <v>0.331787</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>0.234568</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>0.5663549999999999</v>
       </c>
     </row>
@@ -606,12 +652,18 @@
         <v>5423941.581</v>
       </c>
       <c r="D8" t="n">
+        <v>20.604</v>
+      </c>
+      <c r="E8" t="n">
+        <v>20.604</v>
+      </c>
+      <c r="F8" t="n">
         <v>0.316036</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>0.240833</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>0.5568689999999999</v>
       </c>
     </row>
@@ -628,12 +680,18 @@
         <v>5423930.166</v>
       </c>
       <c r="D9" t="n">
+        <v>20.231001</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20.231001</v>
+      </c>
+      <c r="F9" t="n">
         <v>0.247567</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
         <v>0.237406</v>
       </c>
-      <c r="F9" t="n">
+      <c r="H9" t="n">
         <v>0.484973</v>
       </c>
     </row>
@@ -650,12 +708,18 @@
         <v>5423912.414</v>
       </c>
       <c r="D10" t="n">
+        <v>19.983</v>
+      </c>
+      <c r="E10" t="n">
+        <v>19.983</v>
+      </c>
+      <c r="F10" t="n">
         <v>0.203829</v>
       </c>
-      <c r="E10" t="n">
+      <c r="G10" t="n">
         <v>0.237765</v>
       </c>
-      <c r="F10" t="n">
+      <c r="H10" t="n">
         <v>0.441594</v>
       </c>
     </row>
@@ -672,12 +736,18 @@
         <v>5423893.543</v>
       </c>
       <c r="D11" t="n">
+        <v>19.732</v>
+      </c>
+      <c r="E11" t="n">
+        <v>19.732</v>
+      </c>
+      <c r="F11" t="n">
         <v>0.160821</v>
       </c>
-      <c r="E11" t="n">
+      <c r="G11" t="n">
         <v>0.234413</v>
       </c>
-      <c r="F11" t="n">
+      <c r="H11" t="n">
         <v>0.395234</v>
       </c>
     </row>
@@ -694,12 +764,18 @@
         <v>5423881.772</v>
       </c>
       <c r="D12" t="n">
+        <v>19.433001</v>
+      </c>
+      <c r="E12" t="n">
+        <v>19.433001</v>
+      </c>
+      <c r="F12" t="n">
         <v>0.139158</v>
       </c>
-      <c r="E12" t="n">
+      <c r="G12" t="n">
         <v>0.232338</v>
       </c>
-      <c r="F12" t="n">
+      <c r="H12" t="n">
         <v>0.371496</v>
       </c>
     </row>
@@ -716,12 +792,18 @@
         <v>5423865.674</v>
       </c>
       <c r="D13" t="n">
+        <v>18.919001</v>
+      </c>
+      <c r="E13" t="n">
+        <v>18.919001</v>
+      </c>
+      <c r="F13" t="n">
         <v>0.118072</v>
       </c>
-      <c r="E13" t="n">
+      <c r="G13" t="n">
         <v>0.229953</v>
       </c>
-      <c r="F13" t="n">
+      <c r="H13" t="n">
         <v>0.348025</v>
       </c>
     </row>
@@ -738,12 +820,18 @@
         <v>5423847.532</v>
       </c>
       <c r="D14" t="n">
+        <v>18.473</v>
+      </c>
+      <c r="E14" t="n">
+        <v>18.473</v>
+      </c>
+      <c r="F14" t="n">
         <v>0.104907</v>
       </c>
-      <c r="E14" t="n">
+      <c r="G14" t="n">
         <v>0.22924</v>
       </c>
-      <c r="F14" t="n">
+      <c r="H14" t="n">
         <v>0.334147</v>
       </c>
     </row>
@@ -760,12 +848,18 @@
         <v>5423839.069</v>
       </c>
       <c r="D15" t="n">
+        <v>18.273001</v>
+      </c>
+      <c r="E15" t="n">
+        <v>18.273001</v>
+      </c>
+      <c r="F15" t="n">
         <v>0.09851699999999999</v>
       </c>
-      <c r="E15" t="n">
+      <c r="G15" t="n">
         <v>0.228101</v>
       </c>
-      <c r="F15" t="n">
+      <c r="H15" t="n">
         <v>0.326618</v>
       </c>
     </row>
@@ -782,12 +876,18 @@
         <v>5423829.244</v>
       </c>
       <c r="D16" t="n">
+        <v>18.094</v>
+      </c>
+      <c r="E16" t="n">
+        <v>18.094</v>
+      </c>
+      <c r="F16" t="n">
         <v>0.09096799999999999</v>
       </c>
-      <c r="E16" t="n">
+      <c r="G16" t="n">
         <v>0.226493</v>
       </c>
-      <c r="F16" t="n">
+      <c r="H16" t="n">
         <v>0.317461</v>
       </c>
     </row>
@@ -804,12 +904,18 @@
         <v>5423819.079</v>
       </c>
       <c r="D17" t="n">
+        <v>17.516001</v>
+      </c>
+      <c r="E17" t="n">
+        <v>17.516001</v>
+      </c>
+      <c r="F17" t="n">
         <v>0.086273</v>
       </c>
-      <c r="E17" t="n">
+      <c r="G17" t="n">
         <v>0.226092</v>
       </c>
-      <c r="F17" t="n">
+      <c r="H17" t="n">
         <v>0.312365</v>
       </c>
     </row>
@@ -826,12 +932,18 @@
         <v>5423812.404</v>
       </c>
       <c r="D18" t="n">
+        <v>17.434</v>
+      </c>
+      <c r="E18" t="n">
+        <v>17.434</v>
+      </c>
+      <c r="F18" t="n">
         <v>0.082691</v>
       </c>
-      <c r="E18" t="n">
+      <c r="G18" t="n">
         <v>0.225122</v>
       </c>
-      <c r="F18" t="n">
+      <c r="H18" t="n">
         <v>0.307813</v>
       </c>
     </row>
@@ -848,12 +960,18 @@
         <v>5423803.196</v>
       </c>
       <c r="D19" t="n">
+        <v>16.945</v>
+      </c>
+      <c r="E19" t="n">
+        <v>16.945</v>
+      </c>
+      <c r="F19" t="n">
         <v>0.079129</v>
       </c>
-      <c r="E19" t="n">
+      <c r="G19" t="n">
         <v>0.224737</v>
       </c>
-      <c r="F19" t="n">
+      <c r="H19" t="n">
         <v>0.303866</v>
       </c>
     </row>
@@ -870,12 +988,18 @@
         <v>5423795.166</v>
       </c>
       <c r="D20" t="n">
+        <v>16.629999</v>
+      </c>
+      <c r="E20" t="n">
+        <v>16.629999</v>
+      </c>
+      <c r="F20" t="n">
         <v>0.076559</v>
       </c>
-      <c r="E20" t="n">
+      <c r="G20" t="n">
         <v>0.224304</v>
       </c>
-      <c r="F20" t="n">
+      <c r="H20" t="n">
         <v>0.300863</v>
       </c>
     </row>
@@ -892,12 +1016,18 @@
         <v>5423788.919</v>
       </c>
       <c r="D21" t="n">
+        <v>16.528</v>
+      </c>
+      <c r="E21" t="n">
+        <v>16.528</v>
+      </c>
+      <c r="F21" t="n">
         <v>0.074139</v>
       </c>
-      <c r="E21" t="n">
+      <c r="G21" t="n">
         <v>0.223571</v>
       </c>
-      <c r="F21" t="n">
+      <c r="H21" t="n">
         <v>0.29771</v>
       </c>
     </row>
@@ -914,12 +1044,18 @@
         <v>5423782.989</v>
       </c>
       <c r="D22" t="n">
+        <v>16.158001</v>
+      </c>
+      <c r="E22" t="n">
+        <v>16.158001</v>
+      </c>
+      <c r="F22" t="n">
         <v>0.07144200000000001</v>
       </c>
-      <c r="E22" t="n">
+      <c r="G22" t="n">
         <v>0.223822</v>
       </c>
-      <c r="F22" t="n">
+      <c r="H22" t="n">
         <v>0.295264</v>
       </c>
     </row>
@@ -936,12 +1072,18 @@
         <v>5423776.149</v>
       </c>
       <c r="D23" t="n">
+        <v>15.826</v>
+      </c>
+      <c r="E23" t="n">
+        <v>15.826</v>
+      </c>
+      <c r="F23" t="n">
         <v>0.06893100000000001</v>
       </c>
-      <c r="E23" t="n">
+      <c r="G23" t="n">
         <v>0.223279</v>
       </c>
-      <c r="F23" t="n">
+      <c r="H23" t="n">
         <v>0.29221</v>
       </c>
     </row>
@@ -958,12 +1100,18 @@
         <v>5423771.029</v>
       </c>
       <c r="D24" t="n">
+        <v>15.556</v>
+      </c>
+      <c r="E24" t="n">
+        <v>15.556</v>
+      </c>
+      <c r="F24" t="n">
         <v>0.06712600000000001</v>
       </c>
-      <c r="E24" t="n">
+      <c r="G24" t="n">
         <v>0.222898</v>
       </c>
-      <c r="F24" t="n">
+      <c r="H24" t="n">
         <v>0.290024</v>
       </c>
     </row>
@@ -980,12 +1128,18 @@
         <v>5423763.381</v>
       </c>
       <c r="D25" t="n">
+        <v>15.263</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15.263</v>
+      </c>
+      <c r="F25" t="n">
         <v>0.065011</v>
       </c>
-      <c r="E25" t="n">
+      <c r="G25" t="n">
         <v>0.222318</v>
       </c>
-      <c r="F25" t="n">
+      <c r="H25" t="n">
         <v>0.287329</v>
       </c>
     </row>
@@ -1002,12 +1156,18 @@
         <v>5423755.011</v>
       </c>
       <c r="D26" t="n">
+        <v>14.935</v>
+      </c>
+      <c r="E26" t="n">
+        <v>14.935</v>
+      </c>
+      <c r="F26" t="n">
         <v>0.06313299999999999</v>
       </c>
-      <c r="E26" t="n">
+      <c r="G26" t="n">
         <v>0.221822</v>
       </c>
-      <c r="F26" t="n">
+      <c r="H26" t="n">
         <v>0.284955</v>
       </c>
     </row>
@@ -1024,12 +1184,18 @@
         <v>5423745.229</v>
       </c>
       <c r="D27" t="n">
+        <v>14.561</v>
+      </c>
+      <c r="E27" t="n">
+        <v>14.561</v>
+      </c>
+      <c r="F27" t="n">
         <v>0.061826</v>
       </c>
-      <c r="E27" t="n">
+      <c r="G27" t="n">
         <v>0.221555</v>
       </c>
-      <c r="F27" t="n">
+      <c r="H27" t="n">
         <v>0.283381</v>
       </c>
     </row>
@@ -1046,12 +1212,18 @@
         <v>5423735.776</v>
       </c>
       <c r="D28" t="n">
+        <v>14.203</v>
+      </c>
+      <c r="E28" t="n">
+        <v>14.203</v>
+      </c>
+      <c r="F28" t="n">
         <v>0.060161</v>
       </c>
-      <c r="E28" t="n">
+      <c r="G28" t="n">
         <v>0.221097</v>
       </c>
-      <c r="F28" t="n">
+      <c r="H28" t="n">
         <v>0.281258</v>
       </c>
     </row>
@@ -1068,12 +1240,18 @@
         <v>5423728.325</v>
       </c>
       <c r="D29" t="n">
+        <v>13.915</v>
+      </c>
+      <c r="E29" t="n">
+        <v>13.915</v>
+      </c>
+      <c r="F29" t="n">
         <v>0.058523</v>
       </c>
-      <c r="E29" t="n">
+      <c r="G29" t="n">
         <v>0.22056</v>
       </c>
-      <c r="F29" t="n">
+      <c r="H29" t="n">
         <v>0.279083</v>
       </c>
     </row>
@@ -1090,12 +1268,18 @@
         <v>5423720.903</v>
       </c>
       <c r="D30" t="n">
+        <v>13.689</v>
+      </c>
+      <c r="E30" t="n">
+        <v>13.689</v>
+      </c>
+      <c r="F30" t="n">
         <v>0.057046</v>
       </c>
-      <c r="E30" t="n">
+      <c r="G30" t="n">
         <v>0.218033</v>
       </c>
-      <c r="F30" t="n">
+      <c r="H30" t="n">
         <v>0.275079</v>
       </c>
     </row>
@@ -1112,12 +1296,18 @@
         <v>5423713.517</v>
       </c>
       <c r="D31" t="n">
+        <v>13.488</v>
+      </c>
+      <c r="E31" t="n">
+        <v>13.488</v>
+      </c>
+      <c r="F31" t="n">
         <v>0.055731</v>
       </c>
-      <c r="E31" t="n">
+      <c r="G31" t="n">
         <v>0.217547</v>
       </c>
-      <c r="F31" t="n">
+      <c r="H31" t="n">
         <v>0.273278</v>
       </c>
     </row>
@@ -1134,12 +1324,18 @@
         <v>5423704.44</v>
       </c>
       <c r="D32" t="n">
+        <v>13.289</v>
+      </c>
+      <c r="E32" t="n">
+        <v>13.289</v>
+      </c>
+      <c r="F32" t="n">
         <v>0.054448</v>
       </c>
-      <c r="E32" t="n">
+      <c r="G32" t="n">
         <v>0.216792</v>
       </c>
-      <c r="F32" t="n">
+      <c r="H32" t="n">
         <v>0.27124</v>
       </c>
     </row>
@@ -1156,12 +1352,18 @@
         <v>5423696.131</v>
       </c>
       <c r="D33" t="n">
+        <v>13.086</v>
+      </c>
+      <c r="E33" t="n">
+        <v>13.086</v>
+      </c>
+      <c r="F33" t="n">
         <v>0.053288</v>
       </c>
-      <c r="E33" t="n">
+      <c r="G33" t="n">
         <v>0.216127</v>
       </c>
-      <c r="F33" t="n">
+      <c r="H33" t="n">
         <v>0.269415</v>
       </c>
     </row>
@@ -1178,12 +1380,18 @@
         <v>5423689.002</v>
       </c>
       <c r="D34" t="n">
+        <v>12.914</v>
+      </c>
+      <c r="E34" t="n">
+        <v>12.914</v>
+      </c>
+      <c r="F34" t="n">
         <v>0.052243</v>
       </c>
-      <c r="E34" t="n">
+      <c r="G34" t="n">
         <v>0.215508</v>
       </c>
-      <c r="F34" t="n">
+      <c r="H34" t="n">
         <v>0.267751</v>
       </c>
     </row>
@@ -1200,12 +1408,18 @@
         <v>5423682.591</v>
       </c>
       <c r="D35" t="n">
+        <v>12.772</v>
+      </c>
+      <c r="E35" t="n">
+        <v>12.772</v>
+      </c>
+      <c r="F35" t="n">
         <v>0.051314</v>
       </c>
-      <c r="E35" t="n">
+      <c r="G35" t="n">
         <v>0.214931</v>
       </c>
-      <c r="F35" t="n">
+      <c r="H35" t="n">
         <v>0.266245</v>
       </c>
     </row>
@@ -1222,12 +1436,18 @@
         <v>5423675.873</v>
       </c>
       <c r="D36" t="n">
+        <v>12.617</v>
+      </c>
+      <c r="E36" t="n">
+        <v>12.617</v>
+      </c>
+      <c r="F36" t="n">
         <v>0.050535</v>
       </c>
-      <c r="E36" t="n">
+      <c r="G36" t="n">
         <v>0.214439</v>
       </c>
-      <c r="F36" t="n">
+      <c r="H36" t="n">
         <v>0.264974</v>
       </c>
     </row>
@@ -1244,12 +1464,18 @@
         <v>5423669.103</v>
       </c>
       <c r="D37" t="n">
+        <v>12.658</v>
+      </c>
+      <c r="E37" t="n">
+        <v>12.658</v>
+      </c>
+      <c r="F37" t="n">
         <v>0.04952</v>
       </c>
-      <c r="E37" t="n">
+      <c r="G37" t="n">
         <v>0.213551</v>
       </c>
-      <c r="F37" t="n">
+      <c r="H37" t="n">
         <v>0.263071</v>
       </c>
     </row>
@@ -1266,12 +1492,18 @@
         <v>5423662.146</v>
       </c>
       <c r="D38" t="n">
+        <v>12.292</v>
+      </c>
+      <c r="E38" t="n">
+        <v>12.292</v>
+      </c>
+      <c r="F38" t="n">
         <v>0.042929</v>
       </c>
-      <c r="E38" t="n">
+      <c r="G38" t="n">
         <v>0.211208</v>
       </c>
-      <c r="F38" t="n">
+      <c r="H38" t="n">
         <v>0.254137</v>
       </c>
     </row>
@@ -1288,12 +1520,18 @@
         <v>5423666.1</v>
       </c>
       <c r="D39" t="n">
+        <v>12.169</v>
+      </c>
+      <c r="E39" t="n">
+        <v>12.169</v>
+      </c>
+      <c r="F39" t="n">
         <v>0.041881</v>
       </c>
-      <c r="E39" t="n">
+      <c r="G39" t="n">
         <v>0.210513</v>
       </c>
-      <c r="F39" t="n">
+      <c r="H39" t="n">
         <v>0.252394</v>
       </c>
     </row>
@@ -1310,12 +1548,18 @@
         <v>5423670.24</v>
       </c>
       <c r="D40" t="n">
+        <v>12.316</v>
+      </c>
+      <c r="E40" t="n">
+        <v>12.316</v>
+      </c>
+      <c r="F40" t="n">
         <v>0.040654</v>
       </c>
-      <c r="E40" t="n">
+      <c r="G40" t="n">
         <v>0.209475</v>
       </c>
-      <c r="F40" t="n">
+      <c r="H40" t="n">
         <v>0.250129</v>
       </c>
     </row>
@@ -1332,12 +1576,18 @@
         <v>5423663.578</v>
       </c>
       <c r="D41" t="n">
+        <v>12.112</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12.112</v>
+      </c>
+      <c r="F41" t="n">
         <v>0.040381</v>
       </c>
-      <c r="E41" t="n">
+      <c r="G41" t="n">
         <v>0.209162</v>
       </c>
-      <c r="F41" t="n">
+      <c r="H41" t="n">
         <v>0.249543</v>
       </c>
     </row>
@@ -1354,12 +1604,18 @@
         <v>5423654.783</v>
       </c>
       <c r="D42" t="n">
+        <v>11.724</v>
+      </c>
+      <c r="E42" t="n">
+        <v>11.724</v>
+      </c>
+      <c r="F42" t="n">
         <v>0.039571</v>
       </c>
-      <c r="E42" t="n">
+      <c r="G42" t="n">
         <v>0.211416</v>
       </c>
-      <c r="F42" t="n">
+      <c r="H42" t="n">
         <v>0.250987</v>
       </c>
     </row>
@@ -1376,12 +1632,18 @@
         <v>5423646.209</v>
       </c>
       <c r="D43" t="n">
+        <v>11.364</v>
+      </c>
+      <c r="E43" t="n">
+        <v>11.364</v>
+      </c>
+      <c r="F43" t="n">
         <v>0.039069</v>
       </c>
-      <c r="E43" t="n">
+      <c r="G43" t="n">
         <v>0.210382</v>
       </c>
-      <c r="F43" t="n">
+      <c r="H43" t="n">
         <v>0.249451</v>
       </c>
     </row>
@@ -1398,12 +1660,18 @@
         <v>5423637.96</v>
       </c>
       <c r="D44" t="n">
+        <v>11.392</v>
+      </c>
+      <c r="E44" t="n">
+        <v>11.392</v>
+      </c>
+      <c r="F44" t="n">
         <v>0.038481</v>
       </c>
-      <c r="E44" t="n">
+      <c r="G44" t="n">
         <v>0.208753</v>
       </c>
-      <c r="F44" t="n">
+      <c r="H44" t="n">
         <v>0.247234</v>
       </c>
     </row>
@@ -1420,12 +1688,18 @@
         <v>5423630.178</v>
       </c>
       <c r="D45" t="n">
+        <v>11.537</v>
+      </c>
+      <c r="E45" t="n">
+        <v>11.537</v>
+      </c>
+      <c r="F45" t="n">
         <v>0.038064</v>
       </c>
-      <c r="E45" t="n">
+      <c r="G45" t="n">
         <v>0.207043</v>
       </c>
-      <c r="F45" t="n">
+      <c r="H45" t="n">
         <v>0.245107</v>
       </c>
     </row>
@@ -1442,12 +1716,18 @@
         <v>5423623.396</v>
       </c>
       <c r="D46" t="n">
+        <v>12.049</v>
+      </c>
+      <c r="E46" t="n">
+        <v>12.049</v>
+      </c>
+      <c r="F46" t="n">
         <v>0.03725</v>
       </c>
-      <c r="E46" t="n">
+      <c r="G46" t="n">
         <v>0.208955</v>
       </c>
-      <c r="F46" t="n">
+      <c r="H46" t="n">
         <v>0.246205</v>
       </c>
     </row>
@@ -1464,12 +1744,18 @@
         <v>5423605.784</v>
       </c>
       <c r="D47" t="n">
+        <v>12.726</v>
+      </c>
+      <c r="E47" t="n">
+        <v>12.726</v>
+      </c>
+      <c r="F47" t="n">
         <v>0.036582</v>
       </c>
-      <c r="E47" t="n">
+      <c r="G47" t="n">
         <v>0.206321</v>
       </c>
-      <c r="F47" t="n">
+      <c r="H47" t="n">
         <v>0.242903</v>
       </c>
     </row>
@@ -1486,12 +1772,18 @@
         <v>5423578.714</v>
       </c>
       <c r="D48" t="n">
+        <v>13.636</v>
+      </c>
+      <c r="E48" t="n">
+        <v>13.636</v>
+      </c>
+      <c r="F48" t="n">
         <v>0.036332</v>
       </c>
-      <c r="E48" t="n">
+      <c r="G48" t="n">
         <v>0.202915</v>
       </c>
-      <c r="F48" t="n">
+      <c r="H48" t="n">
         <v>0.239247</v>
       </c>
     </row>
@@ -1508,12 +1800,18 @@
         <v>5423570.902</v>
       </c>
       <c r="D49" t="n">
+        <v>14.178</v>
+      </c>
+      <c r="E49" t="n">
+        <v>14.178</v>
+      </c>
+      <c r="F49" t="n">
         <v>0.036215</v>
       </c>
-      <c r="E49" t="n">
+      <c r="G49" t="n">
         <v>0.201214</v>
       </c>
-      <c r="F49" t="n">
+      <c r="H49" t="n">
         <v>0.237429</v>
       </c>
     </row>
@@ -1530,12 +1828,18 @@
         <v>5423549.699</v>
       </c>
       <c r="D50" t="n">
+        <v>14.634</v>
+      </c>
+      <c r="E50" t="n">
+        <v>14.634</v>
+      </c>
+      <c r="F50" t="n">
         <v>0.036649</v>
       </c>
-      <c r="E50" t="n">
+      <c r="G50" t="n">
         <v>0.202861</v>
       </c>
-      <c r="F50" t="n">
+      <c r="H50" t="n">
         <v>0.23951</v>
       </c>
     </row>
@@ -1552,12 +1856,18 @@
         <v>5423533.188</v>
       </c>
       <c r="D51" t="n">
+        <v>15.664</v>
+      </c>
+      <c r="E51" t="n">
+        <v>15.664</v>
+      </c>
+      <c r="F51" t="n">
         <v>0.037059</v>
       </c>
-      <c r="E51" t="n">
+      <c r="G51" t="n">
         <v>0.199738</v>
       </c>
-      <c r="F51" t="n">
+      <c r="H51" t="n">
         <v>0.236797</v>
       </c>
     </row>
@@ -1574,12 +1884,18 @@
         <v>5423533.838</v>
       </c>
       <c r="D52" t="n">
+        <v>16.684</v>
+      </c>
+      <c r="E52" t="n">
+        <v>16.684</v>
+      </c>
+      <c r="F52" t="n">
         <v>0.037365</v>
       </c>
-      <c r="E52" t="n">
+      <c r="G52" t="n">
         <v>0.19725</v>
       </c>
-      <c r="F52" t="n">
+      <c r="H52" t="n">
         <v>0.234615</v>
       </c>
     </row>
@@ -1596,12 +1912,18 @@
         <v>5423534.941</v>
       </c>
       <c r="D53" t="n">
+        <v>17.681999</v>
+      </c>
+      <c r="E53" t="n">
+        <v>17.681999</v>
+      </c>
+      <c r="F53" t="n">
         <v>0.037925</v>
       </c>
-      <c r="E53" t="n">
+      <c r="G53" t="n">
         <v>0.195083</v>
       </c>
-      <c r="F53" t="n">
+      <c r="H53" t="n">
         <v>0.233008</v>
       </c>
     </row>
@@ -1618,12 +1940,18 @@
         <v>5423536.254</v>
       </c>
       <c r="D54" t="n">
+        <v>18.461</v>
+      </c>
+      <c r="E54" t="n">
+        <v>18.461</v>
+      </c>
+      <c r="F54" t="n">
         <v>0.038907</v>
       </c>
-      <c r="E54" t="n">
+      <c r="G54" t="n">
         <v>0.194702</v>
       </c>
-      <c r="F54" t="n">
+      <c r="H54" t="n">
         <v>0.233609</v>
       </c>
     </row>
@@ -1640,12 +1968,18 @@
         <v>5423537.81</v>
       </c>
       <c r="D55" t="n">
+        <v>19.042</v>
+      </c>
+      <c r="E55" t="n">
+        <v>19.042</v>
+      </c>
+      <c r="F55" t="n">
         <v>0.040225</v>
       </c>
-      <c r="E55" t="n">
+      <c r="G55" t="n">
         <v>0.193267</v>
       </c>
-      <c r="F55" t="n">
+      <c r="H55" t="n">
         <v>0.233492</v>
       </c>
     </row>
@@ -1662,12 +1996,18 @@
         <v>5423538.394</v>
       </c>
       <c r="D56" t="n">
+        <v>19.643</v>
+      </c>
+      <c r="E56" t="n">
+        <v>19.643</v>
+      </c>
+      <c r="F56" t="n">
         <v>0.042278</v>
       </c>
-      <c r="E56" t="n">
+      <c r="G56" t="n">
         <v>0.191844</v>
       </c>
-      <c r="F56" t="n">
+      <c r="H56" t="n">
         <v>0.234122</v>
       </c>
     </row>
@@ -1684,12 +2024,18 @@
         <v>5423539.853</v>
       </c>
       <c r="D57" t="n">
+        <v>19.983999</v>
+      </c>
+      <c r="E57" t="n">
+        <v>19.983999</v>
+      </c>
+      <c r="F57" t="n">
         <v>0.044228</v>
       </c>
-      <c r="E57" t="n">
+      <c r="G57" t="n">
         <v>0.190995</v>
       </c>
-      <c r="F57" t="n">
+      <c r="H57" t="n">
         <v>0.235223</v>
       </c>
     </row>
@@ -1706,12 +2052,18 @@
         <v>5423541.02</v>
       </c>
       <c r="D58" t="n">
+        <v>20.039</v>
+      </c>
+      <c r="E58" t="n">
+        <v>20.039</v>
+      </c>
+      <c r="F58" t="n">
         <v>0.047037</v>
       </c>
-      <c r="E58" t="n">
+      <c r="G58" t="n">
         <v>0.191</v>
       </c>
-      <c r="F58" t="n">
+      <c r="H58" t="n">
         <v>0.238037</v>
       </c>
     </row>
@@ -1728,12 +2080,18 @@
         <v>5423542.528</v>
       </c>
       <c r="D59" t="n">
+        <v>20.066</v>
+      </c>
+      <c r="E59" t="n">
+        <v>20.066</v>
+      </c>
+      <c r="F59" t="n">
         <v>0.050317</v>
       </c>
-      <c r="E59" t="n">
+      <c r="G59" t="n">
         <v>0.190592</v>
       </c>
-      <c r="F59" t="n">
+      <c r="H59" t="n">
         <v>0.240909</v>
       </c>
     </row>
@@ -1750,12 +2108,18 @@
         <v>5423543.501</v>
       </c>
       <c r="D60" t="n">
+        <v>20.049</v>
+      </c>
+      <c r="E60" t="n">
+        <v>20.049</v>
+      </c>
+      <c r="F60" t="n">
         <v>0.054991</v>
       </c>
-      <c r="E60" t="n">
+      <c r="G60" t="n">
         <v>0.190264</v>
       </c>
-      <c r="F60" t="n">
+      <c r="H60" t="n">
         <v>0.245255</v>
       </c>
     </row>
@@ -1772,12 +2136,18 @@
         <v>5423544.668</v>
       </c>
       <c r="D61" t="n">
+        <v>19.990999</v>
+      </c>
+      <c r="E61" t="n">
+        <v>19.990999</v>
+      </c>
+      <c r="F61" t="n">
         <v>0.05902</v>
       </c>
-      <c r="E61" t="n">
+      <c r="G61" t="n">
         <v>0.190144</v>
       </c>
-      <c r="F61" t="n">
+      <c r="H61" t="n">
         <v>0.249164</v>
       </c>
     </row>
@@ -1794,12 +2164,18 @@
         <v>5423532.22</v>
       </c>
       <c r="D62" t="n">
+        <v>20.046</v>
+      </c>
+      <c r="E62" t="n">
+        <v>20.046</v>
+      </c>
+      <c r="F62" t="n">
         <v>0.065661</v>
       </c>
-      <c r="E62" t="n">
+      <c r="G62" t="n">
         <v>0.19034</v>
       </c>
-      <c r="F62" t="n">
+      <c r="H62" t="n">
         <v>0.256001</v>
       </c>
     </row>
@@ -1816,12 +2192,18 @@
         <v>5423527.204</v>
       </c>
       <c r="D63" t="n">
+        <v>19.941</v>
+      </c>
+      <c r="E63" t="n">
+        <v>19.941</v>
+      </c>
+      <c r="F63" t="n">
         <v>0.073518</v>
       </c>
-      <c r="E63" t="n">
+      <c r="G63" t="n">
         <v>0.190298</v>
       </c>
-      <c r="F63" t="n">
+      <c r="H63" t="n">
         <v>0.263816</v>
       </c>
     </row>
@@ -1838,12 +2220,18 @@
         <v>5423540.219</v>
       </c>
       <c r="D64" t="n">
+        <v>19.940001</v>
+      </c>
+      <c r="E64" t="n">
+        <v>19.940001</v>
+      </c>
+      <c r="F64" t="n">
         <v>0.082494</v>
       </c>
-      <c r="E64" t="n">
+      <c r="G64" t="n">
         <v>0.190315</v>
       </c>
-      <c r="F64" t="n">
+      <c r="H64" t="n">
         <v>0.272809</v>
       </c>
     </row>
@@ -1860,12 +2248,18 @@
         <v>5423511.1642151</v>
       </c>
       <c r="D65" t="n">
+        <v>20.018</v>
+      </c>
+      <c r="E65" t="n">
+        <v>20.018</v>
+      </c>
+      <c r="F65" t="n">
         <v>0.09715799999999999</v>
       </c>
-      <c r="E65" t="n">
+      <c r="G65" t="n">
         <v>0.189992</v>
       </c>
-      <c r="F65" t="n">
+      <c r="H65" t="n">
         <v>0.28715</v>
       </c>
     </row>
@@ -1882,12 +2276,18 @@
         <v>5423464.549959657</v>
       </c>
       <c r="D66" t="n">
+        <v>20.002001</v>
+      </c>
+      <c r="E66" t="n">
+        <v>20.002001</v>
+      </c>
+      <c r="F66" t="n">
         <v>0.144643</v>
       </c>
-      <c r="E66" t="n">
+      <c r="G66" t="n">
         <v>0.190476</v>
       </c>
-      <c r="F66" t="n">
+      <c r="H66" t="n">
         <v>0.335119</v>
       </c>
     </row>
@@ -1904,12 +2304,18 @@
         <v>5423423.716027891</v>
       </c>
       <c r="D67" t="n">
+        <v>20.167999</v>
+      </c>
+      <c r="E67" t="n">
+        <v>20.167999</v>
+      </c>
+      <c r="F67" t="n">
         <v>0.293752</v>
       </c>
-      <c r="E67" t="n">
+      <c r="G67" t="n">
         <v>0.19128</v>
       </c>
-      <c r="F67" t="n">
+      <c r="H67" t="n">
         <v>0.485032</v>
       </c>
     </row>
@@ -1926,12 +2332,18 @@
         <v>5423348.944608703</v>
       </c>
       <c r="D68" t="n">
+        <v>46.332001</v>
+      </c>
+      <c r="E68" t="n">
+        <v>46.332001</v>
+      </c>
+      <c r="F68" t="n">
         <v>0.38862</v>
       </c>
-      <c r="E68" t="n">
+      <c r="G68" t="n">
         <v>0.18169</v>
       </c>
-      <c r="F68" t="n">
+      <c r="H68" t="n">
         <v>0.57031</v>
       </c>
     </row>
@@ -1948,12 +2360,18 @@
         <v>5423312.76796278</v>
       </c>
       <c r="D69" t="n">
+        <v>91.633003</v>
+      </c>
+      <c r="E69" t="n">
+        <v>91.633003</v>
+      </c>
+      <c r="F69" t="n">
         <v>0.89672</v>
       </c>
-      <c r="E69" t="n">
+      <c r="G69" t="n">
         <v>0.24234</v>
       </c>
-      <c r="F69" t="n">
+      <c r="H69" t="n">
         <v>1.13906</v>
       </c>
     </row>
@@ -1970,12 +2388,18 @@
         <v>5423241.179389093</v>
       </c>
       <c r="D70" t="n">
+        <v>119.489998</v>
+      </c>
+      <c r="E70" t="n">
+        <v>119.489998</v>
+      </c>
+      <c r="F70" t="n">
         <v>1.693565</v>
       </c>
-      <c r="E70" t="n">
+      <c r="G70" t="n">
         <v>0.329467</v>
       </c>
-      <c r="F70" t="n">
+      <c r="H70" t="n">
         <v>2.023032</v>
       </c>
     </row>
@@ -1992,12 +2416,18 @@
         <v>5423249.218</v>
       </c>
       <c r="D71" t="n">
+        <v>122.445</v>
+      </c>
+      <c r="E71" t="n">
+        <v>122.445</v>
+      </c>
+      <c r="F71" t="n">
         <v>1.9137</v>
       </c>
-      <c r="E71" t="n">
+      <c r="G71" t="n">
         <v>0.340762</v>
       </c>
-      <c r="F71" t="n">
+      <c r="H71" t="n">
         <v>2.254462</v>
       </c>
     </row>
@@ -2014,12 +2444,18 @@
         <v>5423228.542</v>
       </c>
       <c r="D72" t="n">
+        <v>104.524002</v>
+      </c>
+      <c r="E72" t="n">
+        <v>104.524002</v>
+      </c>
+      <c r="F72" t="n">
         <v>1.382242</v>
       </c>
-      <c r="E72" t="n">
+      <c r="G72" t="n">
         <v>0.279542</v>
       </c>
-      <c r="F72" t="n">
+      <c r="H72" t="n">
         <v>1.661784</v>
       </c>
     </row>
@@ -2036,12 +2472,18 @@
         <v>5423269.479</v>
       </c>
       <c r="D73" t="n">
+        <v>76.593002</v>
+      </c>
+      <c r="E73" t="n">
+        <v>76.593002</v>
+      </c>
+      <c r="F73" t="n">
         <v>0.802502</v>
       </c>
-      <c r="E73" t="n">
+      <c r="G73" t="n">
         <v>0.214845</v>
       </c>
-      <c r="F73" t="n">
+      <c r="H73" t="n">
         <v>1.017347</v>
       </c>
     </row>
@@ -2058,12 +2500,18 @@
         <v>5423143.827</v>
       </c>
       <c r="D74" t="n">
+        <v>102.750999</v>
+      </c>
+      <c r="E74" t="n">
+        <v>102.750999</v>
+      </c>
+      <c r="F74" t="n">
         <v>1.71337</v>
       </c>
-      <c r="E74" t="n">
+      <c r="G74" t="n">
         <v>0.274704</v>
       </c>
-      <c r="F74" t="n">
+      <c r="H74" t="n">
         <v>1.988074</v>
       </c>
     </row>
@@ -2080,12 +2528,18 @@
         <v>5423095.066</v>
       </c>
       <c r="D75" t="n">
+        <v>47.193001</v>
+      </c>
+      <c r="E75" t="n">
+        <v>47.193001</v>
+      </c>
+      <c r="F75" t="n">
         <v>0.554856</v>
       </c>
-      <c r="E75" t="n">
+      <c r="G75" t="n">
         <v>0.189866</v>
       </c>
-      <c r="F75" t="n">
+      <c r="H75" t="n">
         <v>0.744722</v>
       </c>
     </row>
@@ -2102,12 +2556,18 @@
         <v>5423062.479</v>
       </c>
       <c r="D76" t="n">
+        <v>34.785</v>
+      </c>
+      <c r="E76" t="n">
+        <v>34.785</v>
+      </c>
+      <c r="F76" t="n">
         <v>0.399428</v>
       </c>
-      <c r="E76" t="n">
+      <c r="G76" t="n">
         <v>0.193444</v>
       </c>
-      <c r="F76" t="n">
+      <c r="H76" t="n">
         <v>0.5928720000000001</v>
       </c>
     </row>
@@ -2124,12 +2584,18 @@
         <v>5423120.017</v>
       </c>
       <c r="D77" t="n">
+        <v>54.137001</v>
+      </c>
+      <c r="E77" t="n">
+        <v>54.137001</v>
+      </c>
+      <c r="F77" t="n">
         <v>0.628498</v>
       </c>
-      <c r="E77" t="n">
+      <c r="G77" t="n">
         <v>0.195638</v>
       </c>
-      <c r="F77" t="n">
+      <c r="H77" t="n">
         <v>0.824136</v>
       </c>
     </row>
@@ -2146,12 +2612,18 @@
         <v>5423108.621</v>
       </c>
       <c r="D78" t="n">
+        <v>29.462</v>
+      </c>
+      <c r="E78" t="n">
+        <v>29.462</v>
+      </c>
+      <c r="F78" t="n">
         <v>0.220937</v>
       </c>
-      <c r="E78" t="n">
+      <c r="G78" t="n">
         <v>0.20402</v>
       </c>
-      <c r="F78" t="n">
+      <c r="H78" t="n">
         <v>0.424957</v>
       </c>
     </row>
@@ -2168,12 +2640,18 @@
         <v>5423074.392</v>
       </c>
       <c r="D79" t="n">
+        <v>39.395</v>
+      </c>
+      <c r="E79" t="n">
+        <v>39.395</v>
+      </c>
+      <c r="F79" t="n">
         <v>0.391791</v>
       </c>
-      <c r="E79" t="n">
+      <c r="G79" t="n">
         <v>0.200753</v>
       </c>
-      <c r="F79" t="n">
+      <c r="H79" t="n">
         <v>0.592544</v>
       </c>
     </row>
@@ -2190,12 +2668,18 @@
         <v>5423667.314</v>
       </c>
       <c r="D80" t="n">
+        <v>12.533</v>
+      </c>
+      <c r="E80" t="n">
+        <v>12.533</v>
+      </c>
+      <c r="F80" t="n">
         <v>0.048488</v>
       </c>
-      <c r="E80" t="n">
+      <c r="G80" t="n">
         <v>0.212964</v>
       </c>
-      <c r="F80" t="n">
+      <c r="H80" t="n">
         <v>0.261452</v>
       </c>
     </row>
@@ -2212,12 +2696,18 @@
         <v>5423673.695</v>
       </c>
       <c r="D81" t="n">
+        <v>12.623</v>
+      </c>
+      <c r="E81" t="n">
+        <v>12.623</v>
+      </c>
+      <c r="F81" t="n">
         <v>0.043773</v>
       </c>
-      <c r="E81" t="n">
+      <c r="G81" t="n">
         <v>0.211941</v>
       </c>
-      <c r="F81" t="n">
+      <c r="H81" t="n">
         <v>0.255714</v>
       </c>
     </row>
@@ -2234,12 +2724,18 @@
         <v>5423661.689</v>
       </c>
       <c r="D82" t="n">
+        <v>12.112</v>
+      </c>
+      <c r="E82" t="n">
+        <v>12.112</v>
+      </c>
+      <c r="F82" t="n">
         <v>0.040403</v>
       </c>
-      <c r="E82" t="n">
+      <c r="G82" t="n">
         <v>0.209139</v>
       </c>
-      <c r="F82" t="n">
+      <c r="H82" t="n">
         <v>0.249542</v>
       </c>
     </row>
@@ -2256,12 +2752,18 @@
         <v>5423653.804</v>
       </c>
       <c r="D83" t="n">
+        <v>11.724</v>
+      </c>
+      <c r="E83" t="n">
+        <v>11.724</v>
+      </c>
+      <c r="F83" t="n">
         <v>0.039577</v>
       </c>
-      <c r="E83" t="n">
+      <c r="G83" t="n">
         <v>0.211406</v>
       </c>
-      <c r="F83" t="n">
+      <c r="H83" t="n">
         <v>0.250983</v>
       </c>
     </row>
@@ -2278,12 +2780,18 @@
         <v>5423645.53</v>
       </c>
       <c r="D84" t="n">
+        <v>11.362</v>
+      </c>
+      <c r="E84" t="n">
+        <v>11.362</v>
+      </c>
+      <c r="F84" t="n">
         <v>0.039175</v>
       </c>
-      <c r="E84" t="n">
+      <c r="G84" t="n">
         <v>0.21038</v>
       </c>
-      <c r="F84" t="n">
+      <c r="H84" t="n">
         <v>0.249555</v>
       </c>
     </row>
@@ -2300,12 +2808,18 @@
         <v>5423637.474</v>
       </c>
       <c r="D85" t="n">
+        <v>11.392</v>
+      </c>
+      <c r="E85" t="n">
+        <v>11.392</v>
+      </c>
+      <c r="F85" t="n">
         <v>0.038483</v>
       </c>
-      <c r="E85" t="n">
+      <c r="G85" t="n">
         <v>0.208745</v>
       </c>
-      <c r="F85" t="n">
+      <c r="H85" t="n">
         <v>0.247228</v>
       </c>
     </row>
@@ -2322,12 +2836,18 @@
         <v>5423629.267</v>
       </c>
       <c r="D86" t="n">
+        <v>11.537</v>
+      </c>
+      <c r="E86" t="n">
+        <v>11.537</v>
+      </c>
+      <c r="F86" t="n">
         <v>0.038068</v>
       </c>
-      <c r="E86" t="n">
+      <c r="G86" t="n">
         <v>0.207033</v>
       </c>
-      <c r="F86" t="n">
+      <c r="H86" t="n">
         <v>0.245101</v>
       </c>
     </row>
@@ -2344,12 +2864,18 @@
         <v>5423621.661</v>
       </c>
       <c r="D87" t="n">
+        <v>12.049</v>
+      </c>
+      <c r="E87" t="n">
+        <v>12.049</v>
+      </c>
+      <c r="F87" t="n">
         <v>0.037263</v>
       </c>
-      <c r="E87" t="n">
+      <c r="G87" t="n">
         <v>0.208941</v>
       </c>
-      <c r="F87" t="n">
+      <c r="H87" t="n">
         <v>0.246204</v>
       </c>
     </row>

</xml_diff>